<commit_message>
Fon gecmis arsivini statik parcalara ayir
</commit_message>
<xml_diff>
--- a/app/fonlar/getiri/menkul-kiymet-yatirim-fonlari/data/menkul-kiymet-yatirim-fonlari-getiri.xlsx
+++ b/app/fonlar/getiri/menkul-kiymet-yatirim-fonlari/data/menkul-kiymet-yatirim-fonlari-getiri.xlsx
@@ -19,7 +19,7 @@
     <t>Dışa Aktarım Tarihi:</t>
   </si>
   <si>
-    <t>20.08.2026 10:47:42</t>
+    <t>20.08.2026 11:28:00</t>
   </si>
   <si>
     <t>Toplam Kayıt Sayısı:</t>
@@ -7394,25 +7394,25 @@
         <v>7</v>
       </c>
       <c r="E19" s="7">
-        <v>0</v>
+        <v>0.075839</v>
       </c>
       <c r="F19" s="7">
-        <v>0</v>
+        <v>-0.016712</v>
       </c>
       <c r="G19" s="7">
-        <v>0</v>
+        <v>0.629652</v>
       </c>
       <c r="H19" s="7">
-        <v>0</v>
+        <v>0.8861950000000001</v>
       </c>
       <c r="I19" s="7">
-        <v>0</v>
+        <v>0.894012</v>
       </c>
       <c r="J19" s="7">
-        <v>0</v>
+        <v>1.571344</v>
       </c>
       <c r="K19" s="7">
-        <v>0</v>
+        <v>10.786424</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
@@ -8276,25 +8276,25 @@
         <v>6</v>
       </c>
       <c r="E45" s="7">
-        <v>0</v>
+        <v>0.041004</v>
       </c>
       <c r="F45" s="7">
-        <v>0</v>
+        <v>0.013815</v>
       </c>
       <c r="G45" s="7">
-        <v>0</v>
+        <v>-0.0066549999999999995</v>
       </c>
       <c r="H45" s="7">
-        <v>0</v>
+        <v>0.185561</v>
       </c>
       <c r="I45" s="7">
-        <v>0</v>
+        <v>0.239293</v>
       </c>
       <c r="J45" s="7">
-        <v>0</v>
+        <v>1.0953279999999999</v>
       </c>
       <c r="K45" s="7">
-        <v>0</v>
+        <v>2.995025</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
@@ -8379,25 +8379,25 @@
       </c>
       <c r="D48" s="6"/>
       <c r="E48" s="7">
-        <v>0</v>
+        <v>0.031134</v>
       </c>
       <c r="F48" s="7">
-        <v>0</v>
+        <v>0.049915</v>
       </c>
       <c r="G48" s="7">
-        <v>0</v>
+        <v>0.10315300000000001</v>
       </c>
       <c r="H48" s="7">
-        <v>0</v>
+        <v>0.20228200000000002</v>
       </c>
       <c r="I48" s="7">
-        <v>0</v>
+        <v>0.35519100000000003</v>
       </c>
       <c r="J48" s="7">
-        <v>0</v>
+        <v>2.004654</v>
       </c>
       <c r="K48" s="7">
-        <v>0</v>
+        <v>5.402311999999999</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
@@ -8412,25 +8412,25 @@
       </c>
       <c r="D49" s="6"/>
       <c r="E49" s="7">
-        <v>0</v>
+        <v>0.030728</v>
       </c>
       <c r="F49" s="7">
-        <v>0</v>
+        <v>0.02628</v>
       </c>
       <c r="G49" s="7">
-        <v>0</v>
+        <v>0.052396000000000005</v>
       </c>
       <c r="H49" s="7">
-        <v>0</v>
+        <v>0.17707699999999998</v>
       </c>
       <c r="I49" s="7">
-        <v>0</v>
+        <v>0.32333199999999995</v>
       </c>
       <c r="J49" s="7">
-        <v>0</v>
+        <v>1.821745</v>
       </c>
       <c r="K49" s="7">
-        <v>0</v>
+        <v>5.966201</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
@@ -8447,19 +8447,19 @@
         <v>5</v>
       </c>
       <c r="E50" s="7">
-        <v>0.015024</v>
+        <v>0.015019</v>
       </c>
       <c r="F50" s="7">
-        <v>0.01012</v>
+        <v>0.010115</v>
       </c>
       <c r="G50" s="7">
-        <v>0.017399</v>
+        <v>0.017393000000000002</v>
       </c>
       <c r="H50" s="7">
-        <v>0.015988</v>
+        <v>0.015983</v>
       </c>
       <c r="I50" s="7">
-        <v>0.059644</v>
+        <v>0.059639</v>
       </c>
       <c r="J50" s="7"/>
       <c r="K50" s="7"/>
@@ -10215,10 +10215,10 @@
         <v>3</v>
       </c>
       <c r="E108" s="7">
-        <v>0.029354</v>
+        <v>0.034566</v>
       </c>
       <c r="F108" s="7">
-        <v>0.19112200000000001</v>
+        <v>0.197153</v>
       </c>
       <c r="G108" s="7"/>
       <c r="H108" s="7"/>
@@ -11116,25 +11116,25 @@
         <v>2</v>
       </c>
       <c r="E137" s="7">
-        <v>0.033023</v>
+        <v>0.032965</v>
       </c>
       <c r="F137" s="7">
-        <v>0.10124599999999999</v>
+        <v>0.101183</v>
       </c>
       <c r="G137" s="7">
-        <v>0.207427</v>
+        <v>0.20735900000000002</v>
       </c>
       <c r="H137" s="7">
-        <v>0.268208</v>
+        <v>0.268135</v>
       </c>
       <c r="I137" s="7">
-        <v>0.465062</v>
+        <v>0.464978</v>
       </c>
       <c r="J137" s="7">
-        <v>2.406267</v>
+        <v>2.406073</v>
       </c>
       <c r="K137" s="7">
-        <v>3.949921</v>
+        <v>3.9496390000000003</v>
       </c>
     </row>
     <row r="138" spans="1:11" x14ac:dyDescent="0.25">
@@ -12413,25 +12413,25 @@
         <v>3</v>
       </c>
       <c r="E178" s="7">
-        <v>0.039765999999999996</v>
+        <v>0.039767000000000004</v>
       </c>
       <c r="F178" s="7">
         <v>0.08025299999999999</v>
       </c>
       <c r="G178" s="7">
-        <v>0.131491</v>
+        <v>0.131492</v>
       </c>
       <c r="H178" s="7">
-        <v>0.210837</v>
+        <v>0.210838</v>
       </c>
       <c r="I178" s="7">
-        <v>0.401633</v>
+        <v>0.40163400000000005</v>
       </c>
       <c r="J178" s="7">
-        <v>1.819085</v>
+        <v>1.8190870000000001</v>
       </c>
       <c r="K178" s="7">
-        <v>6.62322</v>
+        <v>6.623226</v>
       </c>
     </row>
     <row r="179" spans="1:11" x14ac:dyDescent="0.25">
@@ -13732,19 +13732,19 @@
         <v>3</v>
       </c>
       <c r="E221" s="7">
-        <v>0.057495000000000004</v>
+        <v>0.066154</v>
       </c>
       <c r="F221" s="7">
-        <v>0.05931</v>
+        <v>0.067984</v>
       </c>
       <c r="G221" s="7">
-        <v>0.12603999999999999</v>
+        <v>0.13526</v>
       </c>
       <c r="H221" s="7">
-        <v>0.253413</v>
+        <v>0.263677</v>
       </c>
       <c r="I221" s="7">
-        <v>0.517171</v>
+        <v>0.529594</v>
       </c>
       <c r="J221" s="7"/>
       <c r="K221" s="7"/>
@@ -16141,25 +16141,25 @@
         <v>5</v>
       </c>
       <c r="E294" s="7">
-        <v>0.024297</v>
+        <v>0.031074</v>
       </c>
       <c r="F294" s="7">
-        <v>0.008631999999999999</v>
+        <v>0.015305</v>
       </c>
       <c r="G294" s="7">
-        <v>0.071387</v>
+        <v>0.078476</v>
       </c>
       <c r="H294" s="7">
-        <v>0.21334499999999998</v>
+        <v>0.221373</v>
       </c>
       <c r="I294" s="7">
-        <v>0.500901</v>
+        <v>0.510832</v>
       </c>
       <c r="J294" s="7">
-        <v>1.831275</v>
+        <v>1.8500079999999999</v>
       </c>
       <c r="K294" s="7">
-        <v>9.207258000000001</v>
+        <v>9.274792999999999</v>
       </c>
     </row>
     <row r="295" spans="1:11" x14ac:dyDescent="0.25">
@@ -16343,22 +16343,22 @@
         <v>5</v>
       </c>
       <c r="E300" s="7">
-        <v>0.041384</v>
+        <v>0.049690000000000005</v>
       </c>
       <c r="F300" s="7">
-        <v>0.024014</v>
+        <v>0.032183</v>
       </c>
       <c r="G300" s="7">
-        <v>0.035496</v>
+        <v>0.043756</v>
       </c>
       <c r="H300" s="7">
-        <v>0.073946</v>
+        <v>0.082513</v>
       </c>
       <c r="I300" s="7">
-        <v>0.20203600000000002</v>
+        <v>0.211624</v>
       </c>
       <c r="J300" s="7">
-        <v>1.531931</v>
+        <v>1.552128</v>
       </c>
       <c r="K300" s="7"/>
     </row>
@@ -16500,22 +16500,22 @@
         <v>7</v>
       </c>
       <c r="E305" s="7">
-        <v>0</v>
+        <v>0.19943100000000002</v>
       </c>
       <c r="F305" s="7">
-        <v>0</v>
+        <v>-0.13478199999999999</v>
       </c>
       <c r="G305" s="7">
-        <v>0</v>
+        <v>-0.11810499999999999</v>
       </c>
       <c r="H305" s="7">
-        <v>0</v>
+        <v>-0.049242999999999995</v>
       </c>
       <c r="I305" s="7">
-        <v>0</v>
+        <v>0.899833</v>
       </c>
       <c r="J305" s="7">
-        <v>0</v>
+        <v>3.472633</v>
       </c>
       <c r="K305" s="7"/>
     </row>
@@ -17827,25 +17827,25 @@
         <v>7</v>
       </c>
       <c r="E346" s="7">
-        <v>0</v>
+        <v>0.18398</v>
       </c>
       <c r="F346" s="7">
-        <v>0</v>
+        <v>-0.12258100000000001</v>
       </c>
       <c r="G346" s="7">
-        <v>0</v>
+        <v>-0.107698</v>
       </c>
       <c r="H346" s="7">
-        <v>0</v>
+        <v>-0.025282</v>
       </c>
       <c r="I346" s="7">
-        <v>0</v>
+        <v>0.895935</v>
       </c>
       <c r="J346" s="7">
-        <v>0</v>
+        <v>3.4192590000000003</v>
       </c>
       <c r="K346" s="7">
-        <v>0</v>
+        <v>11.437071000000001</v>
       </c>
     </row>
     <row r="347" spans="1:11" x14ac:dyDescent="0.25">
@@ -21609,25 +21609,25 @@
         <v>3</v>
       </c>
       <c r="E464" s="7">
-        <v>0</v>
+        <v>0.032925</v>
       </c>
       <c r="F464" s="7">
-        <v>0</v>
+        <v>0.06793199999999999</v>
       </c>
       <c r="G464" s="7">
-        <v>0</v>
+        <v>0.129563</v>
       </c>
       <c r="H464" s="7">
-        <v>0</v>
+        <v>0.203137</v>
       </c>
       <c r="I464" s="7">
-        <v>0</v>
+        <v>0.342943</v>
       </c>
       <c r="J464" s="7">
-        <v>0</v>
+        <v>2.086343</v>
       </c>
       <c r="K464" s="7">
-        <v>0</v>
+        <v>6.019272999999999</v>
       </c>
     </row>
     <row r="465" spans="1:11" x14ac:dyDescent="0.25">
@@ -22316,22 +22316,22 @@
         <v>3</v>
       </c>
       <c r="E485" s="7">
-        <v>0</v>
+        <v>0.038134</v>
       </c>
       <c r="F485" s="7">
-        <v>0</v>
+        <v>0.140396</v>
       </c>
       <c r="G485" s="7">
-        <v>0</v>
+        <v>0.253674</v>
       </c>
       <c r="H485" s="7">
-        <v>0</v>
+        <v>0.346678</v>
       </c>
       <c r="I485" s="7">
-        <v>0</v>
+        <v>0.605386</v>
       </c>
       <c r="J485" s="7">
-        <v>0</v>
+        <v>2.469078</v>
       </c>
       <c r="K485" s="7"/>
     </row>
@@ -22607,22 +22607,22 @@
         <v>5</v>
       </c>
       <c r="E494" s="7">
-        <v>0.059847000000000004</v>
+        <v>0.057725</v>
       </c>
       <c r="F494" s="7">
-        <v>0.099384</v>
+        <v>0.09718299999999999</v>
       </c>
       <c r="G494" s="7">
-        <v>0.359633</v>
+        <v>0.356911</v>
       </c>
       <c r="H494" s="7">
-        <v>0.42633000000000004</v>
+        <v>0.423474</v>
       </c>
       <c r="I494" s="7">
-        <v>0.601757</v>
+        <v>0.5985499999999999</v>
       </c>
       <c r="J494" s="7">
-        <v>2.383007</v>
+        <v>2.376234</v>
       </c>
       <c r="K494" s="7"/>
     </row>
@@ -22832,22 +22832,22 @@
         <v>5</v>
       </c>
       <c r="E501" s="7">
-        <v>0.039682</v>
+        <v>0.042475</v>
       </c>
       <c r="F501" s="7">
-        <v>0.160669</v>
+        <v>0.163786</v>
       </c>
       <c r="G501" s="7">
-        <v>0.311046</v>
+        <v>0.31456700000000004</v>
       </c>
       <c r="H501" s="7">
-        <v>0.39848999999999996</v>
+        <v>0.40224600000000005</v>
       </c>
       <c r="I501" s="7">
-        <v>0.491049</v>
+        <v>0.49505299999999997</v>
       </c>
       <c r="J501" s="7">
-        <v>1.8519040000000002</v>
+        <v>1.859564</v>
       </c>
       <c r="K501" s="7"/>
     </row>
@@ -23766,19 +23766,19 @@
         <v>6</v>
       </c>
       <c r="E531" s="7">
-        <v>0.010714</v>
+        <v>0.010513</v>
       </c>
       <c r="F531" s="7">
-        <v>0.013170999999999999</v>
+        <v>0.012969</v>
       </c>
       <c r="G531" s="7">
-        <v>-0.000136</v>
+        <v>-0.000336</v>
       </c>
       <c r="H531" s="7">
-        <v>-0.007696</v>
+        <v>-0.007894</v>
       </c>
       <c r="I531" s="7">
-        <v>0.027849</v>
+        <v>0.027645</v>
       </c>
       <c r="J531" s="7"/>
       <c r="K531" s="7"/>
@@ -25881,22 +25881,22 @@
         <v>6</v>
       </c>
       <c r="E598" s="7">
-        <v>0.05137800000000001</v>
+        <v>0.058112000000000004</v>
       </c>
       <c r="F598" s="7">
-        <v>0.04771</v>
+        <v>0.05442</v>
       </c>
       <c r="G598" s="7">
-        <v>0.139967</v>
+        <v>0.14726699999999998</v>
       </c>
       <c r="H598" s="7">
-        <v>0.288151</v>
+        <v>0.296401</v>
       </c>
       <c r="I598" s="7">
-        <v>0.41295099999999996</v>
+        <v>0.42200000000000004</v>
       </c>
       <c r="J598" s="7">
-        <v>1.80843</v>
+        <v>1.826417</v>
       </c>
       <c r="K598" s="7"/>
     </row>
@@ -25914,25 +25914,25 @@
         <v>7</v>
       </c>
       <c r="E599" s="7">
-        <v>0.171541</v>
+        <v>0.16625800000000002</v>
       </c>
       <c r="F599" s="7">
-        <v>-0.105057</v>
+        <v>-0.109093</v>
       </c>
       <c r="G599" s="7">
-        <v>-0.08773199999999999</v>
+        <v>-0.091846</v>
       </c>
       <c r="H599" s="7">
-        <v>-0.03932</v>
+        <v>-0.043651999999999996</v>
       </c>
       <c r="I599" s="7">
-        <v>0.8632569999999999</v>
+        <v>0.854854</v>
       </c>
       <c r="J599" s="7">
-        <v>3.616575</v>
+        <v>3.5957549999999996</v>
       </c>
       <c r="K599" s="7">
-        <v>11.957661</v>
+        <v>11.899223999999998</v>
       </c>
     </row>
     <row r="600" spans="1:11" x14ac:dyDescent="0.25">
@@ -26678,22 +26678,22 @@
         <v>5</v>
       </c>
       <c r="E623" s="7">
-        <v>0.01601</v>
+        <v>0.018638</v>
       </c>
       <c r="F623" s="7">
-        <v>0.009598</v>
+        <v>0.012209000000000001</v>
       </c>
       <c r="G623" s="7">
-        <v>0.053308999999999995</v>
+        <v>0.056033</v>
       </c>
       <c r="H623" s="7">
-        <v>0.160153</v>
+        <v>0.163154</v>
       </c>
       <c r="I623" s="7">
-        <v>0.24398499999999998</v>
+        <v>0.24720199999999998</v>
       </c>
       <c r="J623" s="7">
-        <v>1.056545</v>
+        <v>1.061865</v>
       </c>
       <c r="K623" s="7"/>
     </row>
@@ -26996,19 +26996,19 @@
         <v>5</v>
       </c>
       <c r="E633" s="7">
-        <v>0</v>
+        <v>0.031838000000000005</v>
       </c>
       <c r="F633" s="7">
-        <v>0</v>
+        <v>0.09012</v>
       </c>
       <c r="G633" s="7">
-        <v>0</v>
+        <v>0.161535</v>
       </c>
       <c r="H633" s="7">
-        <v>0</v>
+        <v>0.027256999999999997</v>
       </c>
       <c r="I633" s="7">
-        <v>0</v>
+        <v>0.105799</v>
       </c>
       <c r="J633" s="7"/>
       <c r="K633" s="7"/>
@@ -27027,22 +27027,22 @@
         <v>3</v>
       </c>
       <c r="E634" s="7">
-        <v>0</v>
+        <v>-0.013354</v>
       </c>
       <c r="F634" s="7">
-        <v>0</v>
+        <v>0.033815</v>
       </c>
       <c r="G634" s="7">
-        <v>0</v>
+        <v>0.124438</v>
       </c>
       <c r="H634" s="7">
-        <v>0</v>
+        <v>0.15691</v>
       </c>
       <c r="I634" s="7">
-        <v>0</v>
+        <v>0.34756</v>
       </c>
       <c r="J634" s="7">
-        <v>0</v>
+        <v>1.726764</v>
       </c>
       <c r="K634" s="7"/>
     </row>
@@ -28413,25 +28413,25 @@
         <v>5</v>
       </c>
       <c r="E678" s="7">
-        <v>0</v>
+        <v>0.032108</v>
       </c>
       <c r="F678" s="7">
-        <v>0</v>
+        <v>-0.002964</v>
       </c>
       <c r="G678" s="7">
-        <v>0</v>
+        <v>0.000604</v>
       </c>
       <c r="H678" s="7">
-        <v>0</v>
+        <v>0.144178</v>
       </c>
       <c r="I678" s="7">
-        <v>0</v>
+        <v>0.271609</v>
       </c>
       <c r="J678" s="7">
-        <v>0</v>
+        <v>1.606157</v>
       </c>
       <c r="K678" s="7">
-        <v>0</v>
+        <v>6.595646</v>
       </c>
     </row>
     <row r="679" spans="1:11" x14ac:dyDescent="0.25">
@@ -28617,22 +28617,22 @@
         <v>6</v>
       </c>
       <c r="E684" s="7">
-        <v>0.11869199999999999</v>
+        <v>0.11412800000000001</v>
       </c>
       <c r="F684" s="7">
-        <v>0.019796</v>
+        <v>0.015635</v>
       </c>
       <c r="G684" s="7">
-        <v>-0.018259</v>
+        <v>-0.022264</v>
       </c>
       <c r="H684" s="7">
-        <v>0.138463</v>
+        <v>0.133818</v>
       </c>
       <c r="I684" s="7">
-        <v>0.1845</v>
+        <v>0.179667</v>
       </c>
       <c r="J684" s="7">
-        <v>0.812458</v>
+        <v>0.805063</v>
       </c>
       <c r="K684" s="7"/>
     </row>
@@ -28650,22 +28650,22 @@
         <v>3</v>
       </c>
       <c r="E685" s="7">
-        <v>0.036953</v>
+        <v>0.040683</v>
       </c>
       <c r="F685" s="7">
-        <v>0.068737</v>
+        <v>0.07258099999999999</v>
       </c>
       <c r="G685" s="7">
-        <v>0.12591</v>
+        <v>0.12995900000000002</v>
       </c>
       <c r="H685" s="7">
-        <v>0.229212</v>
+        <v>0.23363299999999998</v>
       </c>
       <c r="I685" s="7">
-        <v>0.438665</v>
+        <v>0.443839</v>
       </c>
       <c r="J685" s="7">
-        <v>2.22501</v>
+        <v>2.236609</v>
       </c>
       <c r="K685" s="7"/>
     </row>
@@ -28953,22 +28953,22 @@
         <v>2</v>
       </c>
       <c r="E694" s="7">
-        <v>0.032857</v>
+        <v>0.033972</v>
       </c>
       <c r="F694" s="7">
-        <v>0.10299799999999999</v>
+        <v>0.10418799999999999</v>
       </c>
       <c r="G694" s="7">
-        <v>0.217656</v>
+        <v>0.21897099999999997</v>
       </c>
       <c r="H694" s="7">
-        <v>0.281849</v>
+        <v>0.283232</v>
       </c>
       <c r="I694" s="7">
-        <v>0.486366</v>
+        <v>0.487971</v>
       </c>
       <c r="J694" s="7">
-        <v>2.496137</v>
+        <v>2.499911</v>
       </c>
       <c r="K694" s="7"/>
     </row>
@@ -29246,25 +29246,25 @@
         <v>6</v>
       </c>
       <c r="E703" s="7">
-        <v>0.030713</v>
+        <v>0.030269</v>
       </c>
       <c r="F703" s="7">
-        <v>0.05524</v>
+        <v>0.054786</v>
       </c>
       <c r="G703" s="7">
-        <v>0.098541</v>
+        <v>0.098068</v>
       </c>
       <c r="H703" s="7">
-        <v>0.29291</v>
+        <v>0.292353</v>
       </c>
       <c r="I703" s="7">
-        <v>0.38033900000000004</v>
+        <v>0.379744</v>
       </c>
       <c r="J703" s="7">
-        <v>1.0445579999999999</v>
+        <v>1.043677</v>
       </c>
       <c r="K703" s="7">
-        <v>11.111266</v>
+        <v>11.106048000000001</v>
       </c>
     </row>
     <row r="704" spans="1:11" x14ac:dyDescent="0.25">
@@ -29281,25 +29281,25 @@
         <v>6</v>
       </c>
       <c r="E704" s="7">
-        <v>0.021804999999999998</v>
+        <v>0.019818</v>
       </c>
       <c r="F704" s="7">
-        <v>-0.018938</v>
+        <v>-0.020846</v>
       </c>
       <c r="G704" s="7">
-        <v>-0.000833</v>
+        <v>-0.002777</v>
       </c>
       <c r="H704" s="7">
-        <v>0.191491</v>
+        <v>0.189174</v>
       </c>
       <c r="I704" s="7">
-        <v>0.253379</v>
+        <v>0.250941</v>
       </c>
       <c r="J704" s="7">
-        <v>0.903183</v>
+        <v>0.899481</v>
       </c>
       <c r="K704" s="7">
-        <v>10.062404</v>
+        <v>10.040885</v>
       </c>
     </row>
     <row r="705" spans="1:11" x14ac:dyDescent="0.25">
@@ -29791,19 +29791,19 @@
         <v>4</v>
       </c>
       <c r="E720" s="7">
-        <v>0.053569000000000006</v>
+        <v>0.061848</v>
       </c>
       <c r="F720" s="7">
-        <v>0.106068</v>
+        <v>0.114759</v>
       </c>
       <c r="G720" s="7">
-        <v>0.250507</v>
+        <v>0.260333</v>
       </c>
       <c r="H720" s="7">
-        <v>0.42396500000000004</v>
+        <v>0.435155</v>
       </c>
       <c r="I720" s="7">
-        <v>0.597478</v>
+        <v>0.610031</v>
       </c>
       <c r="J720" s="7"/>
       <c r="K720" s="7"/>
@@ -29888,19 +29888,19 @@
         <v>6</v>
       </c>
       <c r="E723" s="7">
-        <v>0</v>
+        <v>-0.033778</v>
       </c>
       <c r="F723" s="7">
-        <v>0</v>
+        <v>0.311386</v>
       </c>
       <c r="G723" s="7">
-        <v>0</v>
+        <v>0.808395</v>
       </c>
       <c r="H723" s="7">
-        <v>0</v>
+        <v>1.383416</v>
       </c>
       <c r="I723" s="7">
-        <v>0</v>
+        <v>1.902895</v>
       </c>
       <c r="J723" s="7"/>
       <c r="K723" s="7"/>
@@ -30177,19 +30177,19 @@
         <v>6</v>
       </c>
       <c r="E732" s="7">
-        <v>0</v>
+        <v>0.042088</v>
       </c>
       <c r="F732" s="7">
-        <v>0</v>
+        <v>0.399105</v>
       </c>
       <c r="G732" s="7">
-        <v>0</v>
+        <v>0.9154810000000001</v>
       </c>
       <c r="H732" s="7">
-        <v>0</v>
+        <v>1.797183</v>
       </c>
       <c r="I732" s="7">
-        <v>0</v>
+        <v>2.364081</v>
       </c>
       <c r="J732" s="7"/>
       <c r="K732" s="7"/>
@@ -30301,22 +30301,22 @@
         <v>6</v>
       </c>
       <c r="E736" s="7">
-        <v>0.06831000000000001</v>
+        <v>0.066872</v>
       </c>
       <c r="F736" s="7">
-        <v>-0.038083</v>
+        <v>-0.039378</v>
       </c>
       <c r="G736" s="7">
-        <v>0.09735900000000001</v>
+        <v>0.09588200000000001</v>
       </c>
       <c r="H736" s="7">
-        <v>0.272742</v>
+        <v>0.271029</v>
       </c>
       <c r="I736" s="7">
-        <v>0.751345</v>
+        <v>0.7489870000000001</v>
       </c>
       <c r="J736" s="7">
-        <v>2.172646</v>
+        <v>2.168375</v>
       </c>
       <c r="K736" s="7"/>
     </row>
@@ -32531,7 +32531,7 @@
         <v>6</v>
       </c>
       <c r="E808" s="7">
-        <v>0.087786</v>
+        <v>0.088165</v>
       </c>
       <c r="F808" s="7"/>
       <c r="G808" s="7"/>
@@ -33796,19 +33796,19 @@
         <v>5</v>
       </c>
       <c r="E849" s="7">
-        <v>0</v>
+        <v>0.052093</v>
       </c>
       <c r="F849" s="7">
-        <v>0</v>
+        <v>0.19733699999999998</v>
       </c>
       <c r="G849" s="7">
-        <v>0</v>
+        <v>0.43095500000000003</v>
       </c>
       <c r="H849" s="7">
-        <v>0</v>
+        <v>0.44974899999999995</v>
       </c>
       <c r="I849" s="7">
-        <v>0</v>
+        <v>0.535046</v>
       </c>
       <c r="J849" s="7"/>
       <c r="K849" s="7"/>
@@ -34191,19 +34191,19 @@
         <v>4</v>
       </c>
       <c r="E862" s="7">
-        <v>0.053879</v>
+        <v>0.06362</v>
       </c>
       <c r="F862" s="7">
-        <v>0.066432</v>
+        <v>0.076289</v>
       </c>
       <c r="G862" s="7">
-        <v>0.141491</v>
+        <v>0.152042</v>
       </c>
       <c r="H862" s="7">
-        <v>0.257989</v>
+        <v>0.269616</v>
       </c>
       <c r="I862" s="7">
-        <v>0.532023</v>
+        <v>0.546183</v>
       </c>
       <c r="J862" s="7"/>
       <c r="K862" s="7"/>
@@ -34855,22 +34855,22 @@
         <v>3</v>
       </c>
       <c r="E882" s="7">
-        <v>0</v>
+        <v>0.033858</v>
       </c>
       <c r="F882" s="7">
-        <v>0</v>
+        <v>0.093667</v>
       </c>
       <c r="G882" s="7">
-        <v>0</v>
+        <v>0.19206499999999999</v>
       </c>
       <c r="H882" s="7">
-        <v>0</v>
+        <v>0.263702</v>
       </c>
       <c r="I882" s="7">
-        <v>0</v>
+        <v>0.45982599999999996</v>
       </c>
       <c r="J882" s="7">
-        <v>0</v>
+        <v>2.313097</v>
       </c>
       <c r="K882" s="7"/>
     </row>
@@ -35558,25 +35558,25 @@
         <v>6</v>
       </c>
       <c r="E903" s="7">
-        <v>0</v>
+        <v>0.027361</v>
       </c>
       <c r="F903" s="7">
-        <v>0</v>
+        <v>0.019975</v>
       </c>
       <c r="G903" s="7">
-        <v>0</v>
+        <v>0.084749</v>
       </c>
       <c r="H903" s="7">
-        <v>0</v>
+        <v>0.23490100000000003</v>
       </c>
       <c r="I903" s="7">
-        <v>0</v>
+        <v>0.30889099999999997</v>
       </c>
       <c r="J903" s="7">
-        <v>0</v>
+        <v>1.2078470000000001</v>
       </c>
       <c r="K903" s="7">
-        <v>0</v>
+        <v>4.486803</v>
       </c>
     </row>
     <row r="904" spans="1:11" x14ac:dyDescent="0.25">
@@ -35593,22 +35593,22 @@
         <v>4</v>
       </c>
       <c r="E904" s="7">
-        <v>0</v>
+        <v>0.055220000000000005</v>
       </c>
       <c r="F904" s="7">
-        <v>0</v>
+        <v>0.04638</v>
       </c>
       <c r="G904" s="7">
-        <v>0</v>
+        <v>0.087523</v>
       </c>
       <c r="H904" s="7">
-        <v>0</v>
+        <v>0.219772</v>
       </c>
       <c r="I904" s="7">
-        <v>0</v>
+        <v>0.413526</v>
       </c>
       <c r="J904" s="7">
-        <v>0</v>
+        <v>1.738567</v>
       </c>
       <c r="K904" s="7"/>
     </row>
@@ -36150,25 +36150,25 @@
         <v>6</v>
       </c>
       <c r="E921" s="7">
-        <v>0</v>
+        <v>0.126824</v>
       </c>
       <c r="F921" s="7">
-        <v>0</v>
+        <v>-0.030427</v>
       </c>
       <c r="G921" s="7">
-        <v>0</v>
+        <v>-0.05163</v>
       </c>
       <c r="H921" s="7">
-        <v>0</v>
+        <v>0.05025</v>
       </c>
       <c r="I921" s="7">
-        <v>0</v>
+        <v>0.44656199999999996</v>
       </c>
       <c r="J921" s="7">
-        <v>0</v>
+        <v>1.8093469999999998</v>
       </c>
       <c r="K921" s="7">
-        <v>0</v>
+        <v>6.262225</v>
       </c>
     </row>
     <row r="922" spans="1:11" x14ac:dyDescent="0.25">
@@ -37903,22 +37903,22 @@
         <v>2</v>
       </c>
       <c r="E976" s="7">
-        <v>0</v>
+        <v>0.034495</v>
       </c>
       <c r="F976" s="7">
-        <v>0</v>
+        <v>0.091045</v>
       </c>
       <c r="G976" s="7">
-        <v>0</v>
+        <v>0.18922799999999998</v>
       </c>
       <c r="H976" s="7">
-        <v>0</v>
+        <v>0.25810099999999997</v>
       </c>
       <c r="I976" s="7">
-        <v>0</v>
+        <v>0.43737499999999996</v>
       </c>
       <c r="J976" s="7">
-        <v>0</v>
+        <v>1.79216</v>
       </c>
       <c r="K976" s="7"/>
     </row>

</xml_diff>